<commit_message>
chore: sync remaining hardware design assets
</commit_message>
<xml_diff>
--- a/kicad/ELSONIC/POWER_BD_SV3/POWER_BD_SV3_DipPart.xlsx
+++ b/kicad/ELSONIC/POWER_BD_SV3/POWER_BD_SV3_DipPart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_AllData\06_Embedded_Proj\KiCAD\ELSONIC\POWER_BD_SV3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998BCB48-C956-460C-849B-FB0666471474}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3996FF2-0EBC-412C-AA67-A6EE8F2DF113}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30600" yWindow="885" windowWidth="24960" windowHeight="14220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30090" yWindow="690" windowWidth="24960" windowHeight="14220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="POWER_BD_SV2" sheetId="1" r:id="rId1"/>
@@ -449,7 +449,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -627,6 +627,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -889,7 +895,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -900,6 +906,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1332,16 +1344,16 @@
       <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <v>32</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="5" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1384,16 +1396,16 @@
       <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="4">
         <v>34</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H5" s="3">
-        <v>1</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="H5" s="5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1410,56 +1422,56 @@
       <c r="D6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="4">
         <v>35</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H6" s="3">
-        <v>1</v>
-      </c>
-      <c r="I6" s="3" t="s">
+      <c r="H6" s="5">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="2">
-        <v>1</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="C7" s="4">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="4">
         <v>36</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H7" s="3">
-        <v>1</v>
-      </c>
-      <c r="I7" s="3" t="s">
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="4">
         <v>3</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="2">
@@ -1514,16 +1526,16 @@
       <c r="D10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="4">
         <v>39</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="H10" s="3">
-        <v>1</v>
-      </c>
-      <c r="I10" s="3" t="s">
+      <c r="H10" s="5">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1580,16 +1592,16 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
+      <c r="A13" s="4">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="2">
-        <v>1</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F13" s="2">
@@ -1618,16 +1630,16 @@
       <c r="D14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="4">
         <v>43</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="3">
-        <v>1</v>
-      </c>
-      <c r="I14" s="3" t="s">
+      <c r="H14" s="5">
+        <v>1</v>
+      </c>
+      <c r="I14" s="5" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1644,16 +1656,16 @@
       <c r="D15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="4">
         <v>44</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H15" s="3">
-        <v>1</v>
-      </c>
-      <c r="I15" s="3" t="s">
+      <c r="H15" s="5">
+        <v>1</v>
+      </c>
+      <c r="I15" s="5" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1684,80 +1696,80 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
+      <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="2">
-        <v>1</v>
-      </c>
-      <c r="D17" s="3" t="s">
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="4">
         <v>46</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="3">
-        <v>1</v>
-      </c>
-      <c r="I17" s="3" t="s">
+      <c r="H17" s="5">
+        <v>1</v>
+      </c>
+      <c r="I17" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
+      <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="2">
-        <v>1</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="4">
         <v>47</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H18" s="3">
-        <v>1</v>
-      </c>
-      <c r="I18" s="3" t="s">
+      <c r="H18" s="5">
+        <v>1</v>
+      </c>
+      <c r="I18" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
+      <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="2">
-        <v>1</v>
-      </c>
-      <c r="D19" s="3" t="s">
+      <c r="C19" s="4">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="4">
         <v>48</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="H19" s="3">
-        <v>1</v>
-      </c>
-      <c r="I19" s="3" t="s">
+      <c r="H19" s="5">
+        <v>1</v>
+      </c>
+      <c r="I19" s="5" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1842,16 +1854,16 @@
       <c r="I23" s="3"/>
     </row>
     <row r="24" spans="1:9" ht="15.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
+      <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="4">
         <v>3</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="5" t="s">
         <v>48</v>
       </c>
       <c r="F24" s="2">

</xml_diff>